<commit_message>
SK edition: same question wording on Scrollr and in Tiny
Scrollr question under the ? icon now equals the Tiny question (Tiny adds only
the greeting with the quest number). Table regenerated in README and
tiny-otazky-sk.xlsx; quest 06 options carry the hoax/pravda part.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V91vdaXdqZdGzghoT7P96H
</commit_message>
<xml_diff>
--- a/2026/sk/tiny-otazky-sk.xlsx
+++ b/2026/sk/tiny-otazky-sk.xlsx
@@ -433,7 +433,7 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="34" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
@@ -467,7 +467,7 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>Otázka v Tiny</t>
+          <t>Otázka v Tiny (= otázka pod otáznikom na Scrollr + pozdrav)</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
@@ -513,7 +513,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Vitaj v queste číslo 01! Tak čo by si povedal/a… je video generované pomocou AI?</t>
+          <t>Vitaj v queste číslo 01! 🤗 Bolo toto video vytvorené pomocou generatívnej AI? Zvoľ buď áno, čiastočne alebo nie.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Quest 03. Používateľ @jozef-h varuje pred výbuchom v rafinérii Slovnaft v Bratislave. Je to pravda? A ak nie, kde a kedy sa to naozaj stalo a čo tam vybuchlo?</t>
+          <t>Quest 03! Používateľ @jozef-h varuje pred výbuchom v rafinérii Slovnaft v Bratislave. Je to pravda? A ak nie, kde a kedy sa to naozaj stalo a čo tam vybuchlo?</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -689,7 +689,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Čau v queste číslo 05! Dokázal/a si zistiť, aké má Lukas243 heslo do e-mailu?</t>
+          <t>Čau v queste číslo 05! Dokážeš zistiť, aké má Lukas243 heslo do e-mailu?</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -740,24 +740,24 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Október 2021</t>
+          <t>Október 2021, bol to hoax</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Január 2022</t>
+          <t>Január 2022, bol to hoax</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Marec 2022</t>
+          <t>Marec 2022, bola to pravda</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>OZNAČIŤ – podľa vašej tabuľky; odporúčame doplniť k dátumu aj „bol to hoax“</t>
+          <t>A alebo B – označiť podľa skutočného dátumu</t>
         </is>
       </c>
     </row>
@@ -773,7 +773,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Hurá na quest 07! Vieš, či tam @HankaX naozaj bola, alebo ten obrázok ukradla (alebo vygenerovala) a postovala to z domu? A ak ho ukradla, kde bola fotka v skutočnosti odfotená?</t>
+          <t>Hurá na quest 07! Bola tam @HankaX naozaj, alebo ten obrázok ukradla (alebo vygenerovala pomocou AI) a postovala to z domu? A ak ho ukradla, kde bola fotka v skutočnosti odfotená?</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -819,7 +819,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Ahoj v queste číslo 08! Postava Tung Tung Tung Sahur odkazuje na skutočnú tradíciu. Ako sa volá jedlo, na ktoré pri nej ľudia budia susedov, a na aký nástroj pritom tradične búchajú?</t>
+          <t>Ahoj v queste číslo 08! Tralalero Tralalá! Tung Tung Tung niečo… Bombardino Crocodilo + kapučíno. Italian Brainrot v roku 2025 ovládol sociálne siete. Málokto ale vie, že postava Tung Tung Tung Sahur odkazuje na skutočnú tradíciu z konkrétnej krajiny. Ako sa volá jedlo, na ktoré pri tejto tradícii ľudia budia susedov, a na aký nástroj pritom tradične búchajú?</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -861,7 +861,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Ahoj v queste 09! Klasické vyhľadávanie v Obrázkoch Google ti tu nemusí priniesť správne výsledky. Možno to už chce poriadne AI vyhľadávanie (cez nástroj TinEye), pretože sme fotku upravili. Ako si si s tým poradil/a? Kto je speváčka na fotografii a z ktorej krajiny pochádza?</t>
+          <t>Ahoj v queste 09! Kto je speváčka na fotografii a z ktorej krajiny pochádza? Klasické vyhľadávanie v Obrázkoch Google ti tu nemusí priniesť správne výsledky – fotku sme upravili, možno to už chce poriadne AI vyhľadávanie (napríklad nástroj https://tineye.com/).</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Quest 10! Je toto bábätko ďalší AI generovaný slop, alebo je to real?</t>
+          <t>Quest 10! Odhaduje sa, že v roku 2025 prebehlo internetom 8 miliónov deepfakes. To už je celkom číslo, čo? 🤯 Ako je na tom toto bábätko? Je to ďalší AI generovaný slop, alebo je to real?</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Quest 11! Tak čo, zverejnil tento príspevok Peter Sagan na sieti X (bývalý Twitter), alebo nie?</t>
+          <t>Quest 11! Zverejnil Peter Sagan tento príspevok na sieti X (bývalý Twitter), alebo nie?</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Dokážeš zistiť, čo bola hlavná správa na serveri SME.sk 21. mája 2012 o 23:49? Wayback Machine ti nemusí stačiť. Veľké noviny si svoje staré vydania odkladajú aj samy – skús to priamo u nich.</t>
+          <t>Quest 12! Dokážeš zistiť, čo bola hlavná správa na serveri SME.sk 21. mája 2012 o 23:49? Wayback Machine ti nemusí stačiť. Veľké noviny si svoje staré vydania odkladajú aj samy – skús to priamo u nich.</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>OZNAČIŤ – podľa archívu SME (možnosti z vašej tabuľky)</t>
+          <t>označiť podľa archívu SME</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Ahoj v queste 13! Čo myslíš? Bolo slovo Košice vyhľadávané na Slovensku v roku 2025 viac ako slovo Bratislava?</t>
+          <t>Ahoj v queste 13! Čo myslíš? Bolo slovo Košice vyhľadávané na Slovensku v roku 2025 viac ako slovo Bratislava? Overiť to môžeš v nástroji https://trends.google.com/explore</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Quest 15 je pekný, však? Tak čo, ako si si poradil/a?</t>
+          <t>Quest 15 je pekný, však? Človek by povedal, že je to scam. Ako veľmi veríš nám, tvorcom AI olympiády? Vytoč si na stránke iWant výhru a zadaj požadované údaje. Tým získaš heslo, ktoré zadáš do Tiny. Tak čo, ako si si poradil/a?</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">

</xml_diff>